<commit_message>
FEAT :construction: implementacion de roles en pantalla
</commit_message>
<xml_diff>
--- a/static/tickets/Ticket_T-20250709-3.xlsx
+++ b/static/tickets/Ticket_T-20250709-3.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,75 +436,80 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Estado Ticket</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Asunto</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Prioridad</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Solicitante</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Afectado</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Área</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Tipo de Falla</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Service Tag</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Número de Serie</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>IP del Equipo</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Extensión</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Piso</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Datos de Atención</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Comentario del Usuario</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Sugerencias</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Fecha de Registro</t>
         </is>
@@ -518,75 +523,80 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Resuelto</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>preba asunto 2</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>prueba solicitante 2</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>prueba afectado 2</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Area1</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Hardware</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>prueba tag 2</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>prueba numero de serie 2</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>prueba de ip de  equipo</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>prueba de extencion</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>PISO 1</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>prueba de  atencion  2</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>prueba de comentario de usaurio 2</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>prueba de sugerencias 2</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>2025-07-09 00:34:51</t>
         </is>

</xml_diff>